<commit_message>
Add real LUT readback audit and verification
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Firmware/Modules/CalLut/CalLut_Validation.xlsx
+++ b/Firmware/Modules/CalLut/CalLut_Validation.xlsx
@@ -591,7 +591,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q17"/>
+  <dimension ref="A1:Q18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1800,12 +1800,95 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>CL-014</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>LUT_READ بازخوانی واقعی هر دو کانال</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>بالا</t>
+        </is>
+      </c>
+      <c r="D18" s="7" t="inlineStr">
+        <is>
+          <t>رکورد LUT فعال در فلش یا جدول تازه commit شده</t>
+        </is>
+      </c>
+      <c r="E18" s="7" t="inlineStr">
+        <is>
+          <t>از لینک ESP فرمان LUT_READ بفرست و payloadهای LUT_DATA کانال ۱ و ۲ را با آرایه‌های Active مقایسه کن؛ سپس بعد از reset تکرار کن</t>
+        </is>
+      </c>
+      <c r="F18" s="7" t="inlineStr">
+        <is>
+          <t>chainMa/powerMw نقاط فعال، به‌خصوص battery 2</t>
+        </is>
+      </c>
+      <c r="G18" s="7" t="inlineStr">
+        <is>
+          <t>یک درخواست قبل و یک درخواست بعد از reset</t>
+        </is>
+      </c>
+      <c r="H18" s="7" t="inlineStr">
+        <is>
+          <t>LUT_DATA مقدار واقعی هر نقطه را برمی‌گرداند؛ کانال غیرفعال فریم صفرنقطه‌ای می‌دهد؛ دادهٔ ناقص active فرض نمی‌شود</t>
+        </is>
+      </c>
+      <c r="I18" s="7" t="inlineStr">
+        <is>
+          <t>رکورد فلش باید بعد از reset همان نقاط را حفظ کند</t>
+        </is>
+      </c>
+      <c r="J18" s="7" t="inlineStr">
+        <is>
+          <t>تطبیق byte/point با func__CalLut_Points/ChainMa/PowerMw و گزارش mismatch در پنل</t>
+        </is>
+      </c>
+      <c r="K18" s="7" t="inlineStr">
+        <is>
+          <t>Host PASS: 144 check؛ شامل دو فریم واقعی LUT_DATA و آخرین نقطهٔ هر دو کانال؛ برد فیزیکی pending</t>
+        </is>
+      </c>
+      <c r="L18" s="7" t="inlineStr">
+        <is>
+          <t>در انتظار</t>
+        </is>
+      </c>
+      <c r="M18" s="7" t="inlineStr">
+        <is>
+          <t>Host جای اندازه‌گیری برد را نمی‌گیرد؛ فلش و readback روی برد واقعی لازم است</t>
+        </is>
+      </c>
+      <c r="N18" s="7" t="inlineStr">
+        <is>
+          <t>Firmware/Modules/CalLut/Tester/run_host_test_cal_lut.sh</t>
+        </is>
+      </c>
+      <c r="O18" s="7" t="inlineStr">
+        <is>
+          <t>WORKTREE</t>
+        </is>
+      </c>
+      <c r="P18" s="7" t="inlineStr"/>
+      <c r="Q18" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation sqref="L5:L17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="L5:L18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>='فهرست‌ها'!$A$2:$A$6</formula1>
     </dataValidation>
-    <dataValidation sqref="C5:C17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C5:C18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>='فهرست‌ها'!$B$9:$B$11</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Audit zero-point LUT transitions
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Firmware/Modules/CalLut/CalLut_Validation.xlsx
+++ b/Firmware/Modules/CalLut/CalLut_Validation.xlsx
@@ -591,7 +591,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q18"/>
+  <dimension ref="A1:Q19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1853,7 +1853,7 @@
       </c>
       <c r="K18" s="7" t="inlineStr">
         <is>
-          <t>Host PASS: 144 check؛ شامل دو فریم واقعی LUT_DATA و آخرین نقطهٔ هر دو کانال؛ برد فیزیکی pending</t>
+          <t>Host PASS: 159 check؛ شامل دو فریم واقعی LUT_DATA، battery 2 مستقل و transition غیرصفر→صفر؛ برد فیزیکی pending</t>
         </is>
       </c>
       <c r="L18" s="7" t="inlineStr">
@@ -1878,6 +1878,89 @@
       </c>
       <c r="P18" s="7" t="inlineStr"/>
       <c r="Q18" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>CL-015</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>حذف override با صفرنقطه</t>
+        </is>
+      </c>
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>بالا</t>
+        </is>
+      </c>
+      <c r="D19" s="7" t="inlineStr">
+        <is>
+          <t>CL-002 یا رکورد فعال با هر دو کانال</t>
+        </is>
+      </c>
+      <c r="E19" s="7" t="inlineStr">
+        <is>
+          <t>LUT_BEGIN با n1=5 و n2=0، CHUNK فقط کانال ۱، COMMIT با CRC درست؛ سپس reset و LUT_READ</t>
+        </is>
+      </c>
+      <c r="F19" s="7" t="inlineStr">
+        <is>
+          <t>کانال ۱ معتبر؛ کانال ۲ count=0؛ before کانال ۲ غیرصفر و after صفرنقطه‌ای</t>
+        </is>
+      </c>
+      <c r="G19" s="7" t="inlineStr">
+        <is>
+          <t>یک تبادل + یک بوت</t>
+        </is>
+      </c>
+      <c r="H19" s="7" t="inlineStr">
+        <is>
+          <t>commit پذیرفته؛ کانال ۱ حفظ می‌شود و override فلش کانال ۲ حذف می‌شود؛ LUT_DATA کانال ۲ فریم صفرنقطه‌ای مستقل می‌دهد</t>
+        </is>
+      </c>
+      <c r="I19" s="7" t="inlineStr">
+        <is>
+          <t>پینگ‌پنگ و پس از reset</t>
+        </is>
+      </c>
+      <c r="J19" s="7" t="inlineStr">
+        <is>
+          <t>status=0، Active کانال ۱ برقرار، Active کانال ۲=false و مقایسهٔ پنل changed-confirmed؛ CRC/count جای chain/power را نگیرد</t>
+        </is>
+      </c>
+      <c r="K19" s="7" t="inlineStr">
+        <is>
+          <t>Host PASS: 159 check؛ board physical pending</t>
+        </is>
+      </c>
+      <c r="L19" s="7" t="inlineStr">
+        <is>
+          <t>در انتظار</t>
+        </is>
+      </c>
+      <c r="M19" s="7" t="inlineStr">
+        <is>
+          <t>Host جای تست برد را نمی‌گیرد؛ حذف override و ماندگاری پس از reset روی برد واقعی لازم است</t>
+        </is>
+      </c>
+      <c r="N19" s="7" t="inlineStr">
+        <is>
+          <t>Firmware/Modules/CalLut/Tester/run_host_test_cal_lut.sh؛ esp_link_panel/Tester/host_test_scenario_cards.js</t>
+        </is>
+      </c>
+      <c r="O19" s="7" t="inlineStr">
+        <is>
+          <t>WORKTREE</t>
+        </is>
+      </c>
+      <c r="P19" s="7" t="n"/>
+      <c r="Q19" s="7" t="inlineStr">
         <is>
           <t>2026-10-07</t>
         </is>
@@ -1919,6 +2002,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
         <is>
@@ -2330,6 +2414,7 @@
         </is>
       </c>
     </row>
+    <row r="10"/>
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
         <is>
@@ -2360,8 +2445,10 @@
           <t>کل تست‌ها</t>
         </is>
       </c>
-      <c r="B13" s="2" t="n">
-        <v>13</v>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
@@ -2424,7 +2511,7 @@
         </is>
       </c>
       <c r="B17" s="2">
-        <f>IF(13=0,0,COUNTIF('برنامه تست'!L:L,"قبول")/13)</f>
+        <f>IF(15=0,0,COUNTIF('برنامه تست'!L:L,"قبول")/15)</f>
         <v/>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -2433,6 +2520,7 @@
         </is>
       </c>
     </row>
+    <row r="18"/>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
@@ -2500,6 +2588,7 @@
         </is>
       </c>
     </row>
+    <row r="7"/>
     <row r="8">
       <c r="A8" s="9" t="inlineStr">
         <is>
@@ -2554,6 +2643,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="24" customHeight="1">
       <c r="A3" s="11" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Audit calibration readback and reset persistence
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Firmware/Modules/CalLut/CalLut_Validation.xlsx
+++ b/Firmware/Modules/CalLut/CalLut_Validation.xlsx
@@ -591,7 +591,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q19"/>
+  <dimension ref="A1:Q20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1966,12 +1966,95 @@
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>CL-016</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>reset با grant و flush NVM</t>
+        </is>
+      </c>
+      <c r="C20" s="7" t="inlineStr">
+        <is>
+          <t>بالا</t>
+        </is>
+      </c>
+      <c r="D20" s="7" t="inlineStr">
+        <is>
+          <t>commit موفق یا commit صفرنقطه‌ای؛ magic معتبر؛ لینک فعال</t>
+        </is>
+      </c>
+      <c r="E20" s="7" t="inlineStr">
+        <is>
+          <t>پس از commit reset را درخواست کن؛ یک اجرای flush موفق و یک اجرای flush ناموفق/تزریق‌شده را بررسی کن</t>
+        </is>
+      </c>
+      <c r="F20" s="7" t="inlineStr">
+        <is>
+          <t>count=0 معتبر؛ grant commit؛ flush success/failure</t>
+        </is>
+      </c>
+      <c r="G20" s="7" t="inlineStr">
+        <is>
+          <t>حداکثر 15s</t>
+        </is>
+      </c>
+      <c r="H20" s="7" t="inlineStr">
+        <is>
+          <t>zero-point commit بدون active table پذیرفته می‌شود؛ reset فقط با grant commit و flush موفق arm می‌شود؛ flush failure کد CAL_LUT_ST_FLASH می‌دهد و reset انجام نمی‌شود</t>
+        </is>
+      </c>
+      <c r="I20" s="7" t="inlineStr">
+        <is>
+          <t>پس از موفقیت one-shot؛ بعد از flush failure grant برای retry حفظ می‌شود</t>
+        </is>
+      </c>
+      <c r="J20" s="7" t="inlineStr">
+        <is>
+          <t>پس از reset /t و LUT_READ/LUT_DATA تازه، هر دو کانال و persistence با expected برابر؛ هیچ reject/timeout/mismatch موفق گزارش نشود</t>
+        </is>
+      </c>
+      <c r="K20" s="7" t="inlineStr">
+        <is>
+          <t>Host PASS: CalLut=159، parser=14 و NVM؛ تست فیزیکی فلش/ریست/باتری انجام نشده و pending است</t>
+        </is>
+      </c>
+      <c r="L20" s="7" t="inlineStr">
+        <is>
+          <t>در انتظار</t>
+        </is>
+      </c>
+      <c r="M20" s="7" t="inlineStr">
+        <is>
+          <t>Host جای تست فیزیکی برد و fault واقعی NVM را نمی‌گیرد؛ commit zero-point، reset و flush روی برد واقعی تکرار شود</t>
+        </is>
+      </c>
+      <c r="N20" s="7" t="inlineStr">
+        <is>
+          <t>Firmware/Modules/CalLut/Tester/run_host_test_cal_lut.sh؛ Firmware/Modules/EspLink/Tester/run_host_test_nvm.sh؛ Firmware/Modules/EspLink/esp_link.c</t>
+        </is>
+      </c>
+      <c r="O20" s="7" t="inlineStr">
+        <is>
+          <t>WORKTREE</t>
+        </is>
+      </c>
+      <c r="P20" s="7" t="n"/>
+      <c r="Q20" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation sqref="L5:L18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="L5:L20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>='فهرست‌ها'!$A$2:$A$6</formula1>
     </dataValidation>
-    <dataValidation sqref="C5:C18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C5:C20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>='فهرست‌ها'!$B$9:$B$11</formula1>
     </dataValidation>
   </dataValidations>
@@ -1985,7 +2068,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2002,7 +2085,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
         <is>
@@ -2189,6 +2271,33 @@
       <c r="E9" s="7" t="inlineStr">
         <is>
           <t>روش قبلی حذف نشده</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>reset grant و flush NVM</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>magic + commit grant؛ flush NVM پیش از arm</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>flush failure = no reset؛ success = reset one-shot</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>cal_lut.c / esp_link.c / esp_link_nvm.c</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>zero-point commit حتی بدون active table معتبر است</t>
         </is>
       </c>
     </row>
@@ -2414,7 +2523,6 @@
         </is>
       </c>
     </row>
-    <row r="10"/>
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
         <is>
@@ -2447,7 +2555,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -2495,7 +2603,7 @@
         </is>
       </c>
       <c r="B16" s="2">
-        <f>COUNTIF('برنامه تست'!L:L,"در انتظار")</f>
+        <f>IF(16=0,0,COUNTIF('برنامه تست'!L:L,"قبول")/16)</f>
         <v/>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -2520,7 +2628,6 @@
         </is>
       </c>
     </row>
-    <row r="18"/>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
@@ -2588,7 +2695,6 @@
         </is>
       </c>
     </row>
-    <row r="7"/>
     <row r="8">
       <c r="A8" s="9" t="inlineStr">
         <is>
@@ -2643,7 +2749,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="24" customHeight="1">
       <c r="A3" s="11" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Fix signed battery calibration fit and LUT warnings
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Firmware/Modules/CalLut/CalLut_Validation.xlsx
+++ b/Firmware/Modules/CalLut/CalLut_Validation.xlsx
@@ -591,7 +591,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q17"/>
+  <dimension ref="A1:Q20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1800,12 +1800,261 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>CL-014</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>LUT_READ بازخوانی واقعی هر دو کانال</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>بالا</t>
+        </is>
+      </c>
+      <c r="D18" s="7" t="inlineStr">
+        <is>
+          <t>رکورد LUT فعال در فلش یا جدول تازه commit شده</t>
+        </is>
+      </c>
+      <c r="E18" s="7" t="inlineStr">
+        <is>
+          <t>از لینک ESP فرمان LUT_READ بفرست و payloadهای LUT_DATA کانال ۱ و ۲ را با آرایه‌های Active مقایسه کن؛ سپس بعد از reset تکرار کن</t>
+        </is>
+      </c>
+      <c r="F18" s="7" t="inlineStr">
+        <is>
+          <t>chainMa/powerMw نقاط فعال، به‌خصوص battery 2</t>
+        </is>
+      </c>
+      <c r="G18" s="7" t="inlineStr">
+        <is>
+          <t>یک درخواست قبل و یک درخواست بعد از reset</t>
+        </is>
+      </c>
+      <c r="H18" s="7" t="inlineStr">
+        <is>
+          <t>LUT_DATA مقدار واقعی هر نقطه را برمی‌گرداند؛ کانال غیرفعال فریم صفرنقطه‌ای می‌دهد؛ دادهٔ ناقص active فرض نمی‌شود</t>
+        </is>
+      </c>
+      <c r="I18" s="7" t="inlineStr">
+        <is>
+          <t>رکورد فلش باید بعد از reset همان نقاط را حفظ کند</t>
+        </is>
+      </c>
+      <c r="J18" s="7" t="inlineStr">
+        <is>
+          <t>تطبیق byte/point با func__CalLut_Points/ChainMa/PowerMw و گزارش mismatch در پنل</t>
+        </is>
+      </c>
+      <c r="K18" s="7" t="inlineStr">
+        <is>
+          <t>Host PASS: 159 check؛ شامل دو فریم واقعی LUT_DATA، battery 2 مستقل و transition غیرصفر→صفر؛ برد فیزیکی pending</t>
+        </is>
+      </c>
+      <c r="L18" s="7" t="inlineStr">
+        <is>
+          <t>در انتظار</t>
+        </is>
+      </c>
+      <c r="M18" s="7" t="inlineStr">
+        <is>
+          <t>Host جای اندازه‌گیری برد را نمی‌گیرد؛ فلش و readback روی برد واقعی لازم است</t>
+        </is>
+      </c>
+      <c r="N18" s="7" t="inlineStr">
+        <is>
+          <t>Firmware/Modules/CalLut/Tester/run_host_test_cal_lut.sh</t>
+        </is>
+      </c>
+      <c r="O18" s="7" t="inlineStr">
+        <is>
+          <t>WORKTREE</t>
+        </is>
+      </c>
+      <c r="P18" s="7" t="inlineStr"/>
+      <c r="Q18" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>CL-015</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>حذف override با صفرنقطه</t>
+        </is>
+      </c>
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>بالا</t>
+        </is>
+      </c>
+      <c r="D19" s="7" t="inlineStr">
+        <is>
+          <t>CL-002 یا رکورد فعال با هر دو کانال</t>
+        </is>
+      </c>
+      <c r="E19" s="7" t="inlineStr">
+        <is>
+          <t>LUT_BEGIN با n1=5 و n2=0، CHUNK فقط کانال ۱، COMMIT با CRC درست؛ سپس reset و LUT_READ</t>
+        </is>
+      </c>
+      <c r="F19" s="7" t="inlineStr">
+        <is>
+          <t>کانال ۱ معتبر؛ کانال ۲ count=0؛ before کانال ۲ غیرصفر و after صفرنقطه‌ای</t>
+        </is>
+      </c>
+      <c r="G19" s="7" t="inlineStr">
+        <is>
+          <t>یک تبادل + یک بوت</t>
+        </is>
+      </c>
+      <c r="H19" s="7" t="inlineStr">
+        <is>
+          <t>commit پذیرفته؛ کانال ۱ حفظ می‌شود و override فلش کانال ۲ حذف می‌شود؛ LUT_DATA کانال ۲ فریم صفرنقطه‌ای مستقل می‌دهد</t>
+        </is>
+      </c>
+      <c r="I19" s="7" t="inlineStr">
+        <is>
+          <t>پینگ‌پنگ و پس از reset</t>
+        </is>
+      </c>
+      <c r="J19" s="7" t="inlineStr">
+        <is>
+          <t>status=0، Active کانال ۱ برقرار، Active کانال ۲=false و مقایسهٔ پنل changed-confirmed؛ CRC/count جای chain/power را نگیرد</t>
+        </is>
+      </c>
+      <c r="K19" s="7" t="inlineStr">
+        <is>
+          <t>Host PASS: 159 check؛ board physical pending</t>
+        </is>
+      </c>
+      <c r="L19" s="7" t="inlineStr">
+        <is>
+          <t>در انتظار</t>
+        </is>
+      </c>
+      <c r="M19" s="7" t="inlineStr">
+        <is>
+          <t>Host جای تست برد را نمی‌گیرد؛ حذف override و ماندگاری پس از reset روی برد واقعی لازم است</t>
+        </is>
+      </c>
+      <c r="N19" s="7" t="inlineStr">
+        <is>
+          <t>Firmware/Modules/CalLut/Tester/run_host_test_cal_lut.sh؛ esp_link_panel/Tester/host_test_scenario_cards.js</t>
+        </is>
+      </c>
+      <c r="O19" s="7" t="inlineStr">
+        <is>
+          <t>WORKTREE</t>
+        </is>
+      </c>
+      <c r="P19" s="7" t="n"/>
+      <c r="Q19" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>CL-016</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>reset با grant و flush NVM</t>
+        </is>
+      </c>
+      <c r="C20" s="7" t="inlineStr">
+        <is>
+          <t>بالا</t>
+        </is>
+      </c>
+      <c r="D20" s="7" t="inlineStr">
+        <is>
+          <t>commit موفق یا commit صفرنقطه‌ای؛ magic معتبر؛ لینک فعال</t>
+        </is>
+      </c>
+      <c r="E20" s="7" t="inlineStr">
+        <is>
+          <t>پس از commit reset را درخواست کن؛ یک اجرای flush موفق و یک اجرای flush ناموفق/تزریق‌شده را بررسی کن</t>
+        </is>
+      </c>
+      <c r="F20" s="7" t="inlineStr">
+        <is>
+          <t>count=0 معتبر؛ grant commit؛ flush success/failure</t>
+        </is>
+      </c>
+      <c r="G20" s="7" t="inlineStr">
+        <is>
+          <t>حداکثر 15s</t>
+        </is>
+      </c>
+      <c r="H20" s="7" t="inlineStr">
+        <is>
+          <t>zero-point commit بدون active table پذیرفته می‌شود؛ reset فقط با grant commit و flush موفق arm می‌شود؛ flush failure کد CAL_LUT_ST_FLASH می‌دهد و reset انجام نمی‌شود</t>
+        </is>
+      </c>
+      <c r="I20" s="7" t="inlineStr">
+        <is>
+          <t>پس از موفقیت one-shot؛ بعد از flush failure grant برای retry حفظ می‌شود</t>
+        </is>
+      </c>
+      <c r="J20" s="7" t="inlineStr">
+        <is>
+          <t>پس از reset /t و LUT_READ/LUT_DATA تازه، هر دو کانال و persistence با expected برابر؛ هیچ reject/timeout/mismatch موفق گزارش نشود</t>
+        </is>
+      </c>
+      <c r="K20" s="7" t="inlineStr">
+        <is>
+          <t>Host PASS: CalLut=159، parser=14 و NVM؛ تست فیزیکی فلش/ریست/باتری انجام نشده و pending است</t>
+        </is>
+      </c>
+      <c r="L20" s="7" t="inlineStr">
+        <is>
+          <t>در انتظار</t>
+        </is>
+      </c>
+      <c r="M20" s="7" t="inlineStr">
+        <is>
+          <t>Host جای تست فیزیکی برد و fault واقعی NVM را نمی‌گیرد؛ commit zero-point، reset و flush روی برد واقعی تکرار شود</t>
+        </is>
+      </c>
+      <c r="N20" s="7" t="inlineStr">
+        <is>
+          <t>Firmware/Modules/CalLut/Tester/run_host_test_cal_lut.sh؛ Firmware/Modules/EspLink/Tester/run_host_test_nvm.sh؛ Firmware/Modules/EspLink/esp_link.c</t>
+        </is>
+      </c>
+      <c r="O20" s="7" t="inlineStr">
+        <is>
+          <t>WORKTREE</t>
+        </is>
+      </c>
+      <c r="P20" s="7" t="n"/>
+      <c r="Q20" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation sqref="L5:L17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="L5:L20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>='فهرست‌ها'!$A$2:$A$6</formula1>
     </dataValidation>
-    <dataValidation sqref="C5:C17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C5:C20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>='فهرست‌ها'!$B$9:$B$11</formula1>
     </dataValidation>
   </dataValidations>
@@ -1819,7 +2068,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2022,6 +2271,33 @@
       <c r="E9" s="7" t="inlineStr">
         <is>
           <t>روش قبلی حذف نشده</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>reset grant و flush NVM</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>magic + commit grant؛ flush NVM پیش از arm</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>flush failure = no reset؛ success = reset one-shot</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>cal_lut.c / esp_link.c / esp_link_nvm.c</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>zero-point commit حتی بدون active table معتبر است</t>
         </is>
       </c>
     </row>
@@ -2277,8 +2553,10 @@
           <t>کل تست‌ها</t>
         </is>
       </c>
-      <c r="B13" s="2" t="n">
-        <v>13</v>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
@@ -2325,7 +2603,7 @@
         </is>
       </c>
       <c r="B16" s="2">
-        <f>COUNTIF('برنامه تست'!L:L,"در انتظار")</f>
+        <f>IF(16=0,0,COUNTIF('برنامه تست'!L:L,"قبول")/16)</f>
         <v/>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -2341,7 +2619,7 @@
         </is>
       </c>
       <c r="B17" s="2">
-        <f>IF(13=0,0,COUNTIF('برنامه تست'!L:L,"قبول")/13)</f>
+        <f>IF(15=0,0,COUNTIF('برنامه تست'!L:L,"قبول")/15)</f>
         <v/>
       </c>
       <c r="C17" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Review: remove stale compiled-table claims (fallback is gain/offset line), escape imported sample fields in panel table (XSS), fix Measurement README power wording, CalLut validation workbook text
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Firmware/Modules/CalLut/CalLut_Validation.xlsx
+++ b/Firmware/Modules/CalLut/CalLut_Validation.xlsx
@@ -555,7 +555,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>جدول‌های کامپایل‌تایم calibration.h می‌مانند و پشتیبان‌اند: فقط وقتی رکورد معتبر در فلش باشد از آن استفاده می‌شود.</t>
+          <t>جدول کامپایل‌شده وجود ندارد. وقتی رکورد معتبر در فلش نباشد، خط گین و آفست (پیش‌فرض گین 3000، آفست 0) استفاده می‌شود؛ وقتی رکورد معتبر در فلش باشد از آن استفاده می‌شود.</t>
         </is>
       </c>
     </row>
@@ -759,7 +759,7 @@
       </c>
       <c r="H5" s="7" t="inlineStr">
         <is>
-          <t>func__CalLut_Active هر دو کانال false؛ مسیر اندازه‌گیری از جدول calibration.h استفاده می‌کند</t>
+          <t>func__CalLut_Active هر دو کانال false؛ مسیر اندازه‌گیری از خط گین و آفست استفاده می‌کند</t>
         </is>
       </c>
       <c r="I5" s="7" t="inlineStr">
@@ -1765,7 +1765,7 @@
       </c>
       <c r="J17" s="7" t="inlineStr">
         <is>
-          <t>Active=false و خوانش‌ها برابر جدول calibration.h</t>
+          <t>Active=false و خوانش‌ها برابر خط گین و آفست</t>
         </is>
       </c>
       <c r="K17" s="7" t="inlineStr">
@@ -2255,7 +2255,7 @@
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>جدول‌های calibration.h</t>
+          <t>جدول‌های فلش (CalLut) و خط گین و آفست</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">

</xml_diff>

<commit_message>
validation: update all Excels for v1.87 panel styled dialogs (#pmod queue Enter/Esc) + task_control snapshot zeroing (2026-10-12)
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Firmware/Modules/CalLut/CalLut_Validation.xlsx
+++ b/Firmware/Modules/CalLut/CalLut_Validation.xlsx
@@ -591,7 +591,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q20"/>
+  <dimension ref="A1:Q21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -2046,6 +2046,76 @@
       <c r="Q20" s="7" t="inlineStr">
         <is>
           <t>2026-10-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>CL-020</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>پنل دیالوگ LUT</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>متوسط</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>پنل وصل + LUT آماده</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>از پنل LUT را push کن؛ دیالوگ تأیید ریست باید با کادر تیره همرنگ پنل بیاید و Enter تأیید و Esc لغو کند</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>LUT 2 کانال</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>10s</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>دیالوگ با استایل #pmod/#121a2c، بدون alert سفید ویندوز؛ Enter=تأیید Esc=انصراف؛ صف PMQ یکی‌یکی</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>دیالوگ تیره + Enter/Esc کار کند</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>نیاز به تکرار</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr"/>
+      <c r="N21" t="inlineStr"/>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>62f3782</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr"/>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(validation): write test-sheet numbers in decimal, not hex
Per user order (tests must read for a human): the only 5 hex cells in
the برنامه تست sheets converted - 0xFFFF->65535, fault=0x3F->63,
commands 0x30/0x31->48/49 with their names, fault 0x40->64 (panel
display noted). Gates green.

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Firmware/Modules/CalLut/CalLut_Validation.xlsx
+++ b/Firmware/Modules/CalLut/CalLut_Validation.xlsx
@@ -749,7 +749,7 @@
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>فلش LUT خالی (0xFFFF)</t>
+          <t>فلش LUT خالی (65535 = خانهٔ پاک‌شدهٔ فلش)</t>
         </is>
       </c>
       <c r="G5" s="7" t="inlineStr">
@@ -2105,14 +2105,11 @@
           <t>نیاز به تکرار</t>
         </is>
       </c>
-      <c r="M21" t="inlineStr"/>
-      <c r="N21" t="inlineStr"/>
       <c r="O21" t="inlineStr">
         <is>
           <t>62f3782</t>
         </is>
       </c>
-      <c r="P21" t="inlineStr"/>
       <c r="Q21" t="inlineStr">
         <is>
           <t>2026-10-12</t>

</xml_diff>

<commit_message>
docs(validation): rewrite every test method step by step
All 240 rows in the 14 validation workbooks now run 'گام ۱..' style:
preparation, exact action, what to watch, and the pass line - written
for a person at the bench, decimal numbers, FAULT_* names. Only the
روش column was rewritten; preconditions, expected behaviour,
acceptance criteria and statuses are the pre-existing ones.

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Firmware/Modules/CalLut/CalLut_Validation.xlsx
+++ b/Firmware/Modules/CalLut/CalLut_Validation.xlsx
@@ -744,7 +744,10 @@
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>برد را بدون هیچ push جدول روشن کن و جریان خوانده‌شده را با جدول کامپایل‌شده مقایسه کن</t>
+          <t>گام ۱: مطمئن شو هیچ جدولی از پنل فرستاده نشده و فلش LUT خالی است (همهٔ خانه‌ها 65535).
+گام ۲: برد را روشن کن و صبر کن بوت کامل شود.
+گام ۳: از پنل ببین هر دو کانال جدول فعال ندارند (Active هر دو false است).
+گام ۴: جریان خوانده‌شدهٔ هر دو کانال را با همان بردی که ماژول LUT نداشت مقایسه کن؛ باید دقیقاً یکی باشد، چون مسیر اندازه‌گیری از خط گین و آفست استفاده می‌کند.</t>
         </is>
       </c>
       <c r="F5" s="7" t="inlineStr">
@@ -827,7 +830,11 @@
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>از پنل یک جدول ۱۷..۲۱ نقطه‌ای برای کانال ۱ بفرست و commit کن</t>
+          <t>گام ۱: لینک ESP را وصل کن و پنل را باز کن.
+گام ۲: برای کانال ۱ یک جدول 17 تا 21 نقطه‌ای بساز و ارسال کن (اول LUT_BEGIN، بعد چانک‌ها، در آخر COMMIT).
+گام ۳: پاسخ برد را بخوان: وضعیت باید 0 باشد (CAL_LUT_ST_OK).
+گام ۴: CRC32 جدول در پنل و CRC32 گزارش‌شدهٔ برد را مقایسه کن؛ باید برابر باشند.
+گام ۵: فرمان LUT_RESET را بفرست و بعد از بالا آمدن برد ببین جدول کانال ۱ فعال شده است (Active = true).</t>
         </is>
       </c>
       <c r="F6" s="7" t="inlineStr">
@@ -910,7 +917,10 @@
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>برق برد را کاملاً قطع و وصل کن (نه ریست نرم)</t>
+          <t>گام ۱: اول تست CL-002 را قبول کن تا یک جدول سالم روی برد فعال باشد و CRC32 آن را یادداشت کن.
+گام ۲: تغذیهٔ برد را کاملاً قطع کن (فقط ریست نرم کافی نیست) و دوباره وصل کن.
+گام ۳: بعد از بوت، CRC32 جدول فعال را از برد بخوان و با مقدار یادداشت‌شده مقایسه کن.
+گام ۴: قطع و وصل کامل را 3 بار تکرار کن؛ هر سه بار CRC32 باید همان مقدار قبلی باشد.</t>
         </is>
       </c>
       <c r="F7" s="7" t="inlineStr">
@@ -993,7 +1003,10 @@
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>عمداً CRC32 اشتباه در LUT_COMMIT بفرست</t>
+          <t>گام ۱: لینک ESP را وصل کن و CRC32 جدول فعال فعلی را یادداشت کن.
+گام ۲: یک جدول بفرست ولی در مرحلهٔ COMMIT عمداً CRC32 اشتباه بده (با CRC واقعی جدول یکی نباشد).
+گام ۳: پاسخ برد را بخوان: وضعیت باید 6 باشد (CAL_LUT_ST_CRC) و commit رد شود.
+گام ۴: CRC32 جدول فعال را دوباره بخوان؛ باید با گام ۱ یکی باشد، یعنی فلش دست‌نخورده مانده است.</t>
         </is>
       </c>
       <c r="F8" s="7" t="inlineStr">
@@ -1076,7 +1089,10 @@
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>جدولی بفرست که محور زنجیره صعودی اکید نیست</t>
+          <t>گام ۱: لینک ESP را وصل کن.
+گام ۲: جدولی بساز که محور زنجیره‌اش (ChainMa) صعودیِ اکید نباشد؛ مثلاً یک نقطهٔ تکراری یا یک نقطه کمتر از قبلی بگذار.
+گام ۳: جدول را کامل بفرست و COMMIT کن.
+گام ۴: پاسخ برد را بخوان: وضعیت باید 4 باشد (CAL_LUT_ST_CHAIN) و جدول نباید فعال شود.</t>
         </is>
       </c>
       <c r="F9" s="7" t="inlineStr">
@@ -1159,7 +1175,10 @@
       </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
-          <t>جدولی بفرست که جریان باتری آن در یک نقطه کم‌تر از نقطهٔ قبلی باشد</t>
+          <t>گام ۱: لینک ESP را وصل کن.
+گام ۲: جدولی بساز که جریان باتری در یکی از نقطه‌ها از نقطهٔ قبلی کمتر باشد (افت داشته باشد).
+گام ۳: جدول را کامل بفرست و COMMIT کن.
+گام ۴: پاسخ برد را بخوان: وضعیت باید 5 باشد (CAL_LUT_ST_DIP) و جدول نباید فعال شود.</t>
         </is>
       </c>
       <c r="F10" s="7" t="inlineStr">
@@ -1242,7 +1261,10 @@
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>یک‌بار با ۱ نقطه و یک‌بار با ۲۵ نقطه commit کن</t>
+          <t>گام ۱: لینک ESP را وصل کن.
+گام ۲: یک جدول فقط با 1 نقطه بفرست و COMMIT کن؛ پاسخ را بخوان.
+گام ۳: یک جدول با 25 نقطه بفرست و COMMIT کن؛ پاسخ را بخوان.
+گام ۴: هر دو بار وضعیت باید 2 باشد (CAL_LUT_ST_COUNT)، چون تعداد نقطهٔ مجاز 2 تا 24 است.</t>
         </is>
       </c>
       <c r="F11" s="7" t="inlineStr">
@@ -1325,7 +1347,10 @@
       </c>
       <c r="E12" s="7" t="inlineStr">
         <is>
-          <t>یک CHUNK را عمداً نفرست و commit کن</t>
+          <t>گام ۱: لینک ESP را وصل کن و یک جدول چندچانکه آماده کن.
+گام ۲: همهٔ چانک‌ها را بفرست به‌جز یکی؛ عمداً یک چانک را نفرست.
+گام ۳: COMMIT را بفرست.
+گام ۴: پاسخ برد را بخوان: وضعیت باید 3 باشد (CAL_LUT_ST_MISSING) و هیچ جدولی فعال نشود.</t>
         </is>
       </c>
       <c r="F12" s="7" t="inlineStr">
@@ -1408,7 +1433,9 @@
       </c>
       <c r="E13" s="7" t="inlineStr">
         <is>
-          <t>بدون LUT_BEGIN مستقیم COMMIT بفرست</t>
+          <t>گام ۱: لینک ESP را وصل کن.
+گام ۲: بدون اینکه LUT_BEGIN بفرستی، مستقیم COMMIT بفرست.
+گام ۳: پاسخ برد را بخوان: وضعیت باید 1 باشد (CAL_LUT_ST_NO_STAGE) و هیچ اتفاقی برای جدول فعال نیفتد.</t>
         </is>
       </c>
       <c r="F13" s="7" t="inlineStr">
@@ -1491,7 +1518,10 @@
       </c>
       <c r="E14" s="7" t="inlineStr">
         <is>
-          <t>در لحظهٔ commit تغذیه را قطع کن؛ چند بار تکرار</t>
+          <t>گام ۱: اول یک جدول سالم commit کن (CL-002) و CRC32 آن را یادداشت کن.
+گام ۲: یک جدول تازه بفرست و دقیقاً وسط COMMIT (موقع پاک/نوشتن فلش) تغذیهٔ برد را قطع کن.
+گام ۳: تغذیه را وصل کن و بعد از بوت، جدول فعال و CRC32 آن را بخوان: یا باید جدول قبلی سالم باشد یا جدول جدید کامل نشسته باشد؛ حالت سوم (نیمه‌کاره) هرگز نباید دیده شود.
+گام ۴: این کار را 5 بار تکرار کن و هر بار بعد از بوت سالم‌بودن رکورد فعال (RecordValidate = true) را بررسی کن.</t>
         </is>
       </c>
       <c r="F14" s="7" t="inlineStr">
@@ -1574,7 +1604,10 @@
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
-          <t>پارامترها را تغییر و ذخیره کن، سپس یک جدول کامل push کن و برعکس</t>
+          <t>گام ۱: چند پارامتر را از پنل از مقدار پیش‌فرض تغییر بده و ذخیره کن؛ مقدارها را یادداشت کن.
+گام ۲: یک جدول LUT کامل push کن و commit کن.
+گام ۳: دوباره یک پارامتر را تغییر و ذخیره کن و یک جدول دیگر push کن (هر دو مسیر ذخیره پشت سر هم).
+گام ۴: برد را ری‌استارت کن و همهٔ پارامترها و جدول را بخوان؛ هیچ‌کدام نباید دیگری را خراب کرده باشد و همه باید با مقدارهای یادداشت‌شده یکی باشند.</t>
         </is>
       </c>
       <c r="F15" s="7" t="inlineStr">
@@ -1657,7 +1690,10 @@
       </c>
       <c r="E16" s="7" t="inlineStr">
         <is>
-          <t>حین BULK فعال، LUT_RESET بفرست</t>
+          <t>گام ۱: یک جدول فعال کن و شارژ را در حالت BULK راه بینداز تا کانال در حال شارژ PWM داشته باشد.
+گام ۲: اسیلوسکوپ را روی گیت همان کانال بگذار.
+گام ۳: حین شارژ فرمان LUT_RESET را بفرست.
+گام ۴: روی اسکوپ ببین که پیش از ریست، duty اول صفر شده و شارژر idle شده باشد؛ ریست نباید وسط پالس اتفاق بیفتد.</t>
         </is>
       </c>
       <c r="F16" s="7" t="inlineStr">
@@ -1740,7 +1776,10 @@
       </c>
       <c r="E17" s="7" t="inlineStr">
         <is>
-          <t>CAL_LUT_VERSION را بالا ببر و فرم‌ور جدید را فلش کن</t>
+          <t>گام ۱: روی برد یک رکورد LUT معتبر با نسخهٔ 1 داشته باش (قبلاً commit شده باشد).
+گام ۲: ثابت CAL_LUT_VERSION را در کد بالا ببر و فرم‌ور جدید را روی همان برد فلش کن.
+گام ۳: برد را بوت کن و وضعیت جدول فعال را بخوان.
+گام ۴: باید جدول فعال نباشد (Active = false) و خوانش جریان به جدول کامپایل‌شده (خط گین و آفست) برگشته باشد.</t>
         </is>
       </c>
       <c r="F17" s="7" t="inlineStr">
@@ -1823,7 +1862,10 @@
       </c>
       <c r="E18" s="7" t="inlineStr">
         <is>
-          <t>از لینک ESP فرمان LUT_READ بفرست و payloadهای LUT_DATA کانال ۱ و ۲ را با آرایه‌های Active مقایسه کن؛ سپس بعد از reset تکرار کن</t>
+          <t>گام ۱: یک جدول فعال روی فلش داشته باش (یا تازه commit کن) و نقاط هر دو کانال را از پنل یادداشت کن.
+گام ۲: از لینک ESP فرمان LUT_READ بفرست.
+گام ۳: داده‌های برگشتی (LUT_DATA کانال ۱ و ۲) را نقطه‌به‌نقطه با نقاط فعال مقایسه کن؛ کانال بدون جدول باید فریم صفرنقطه‌ای بدهد.
+گام ۴: برد را ریست کن و گام ۲ و ۳ را تکرار کن؛ دادهٔ ناقص نباید «فعال» فرض شود و پنل باید هر عدم تطابق (mismatch) را گزارش کند.</t>
         </is>
       </c>
       <c r="F18" s="7" t="inlineStr">
@@ -1906,7 +1948,11 @@
       </c>
       <c r="E19" s="7" t="inlineStr">
         <is>
-          <t>LUT_BEGIN با n1=5 و n2=0، CHUNK فقط کانال ۱، COMMIT با CRC درست؛ سپس reset و LUT_READ</t>
+          <t>گام ۱: از قبل روی هر دو کانال جدول فعال داشته باش (CL-002 برای هر دو) و نقاط کانال ۲ را یادداشت کن.
+گام ۲: LUT_BEGIN را با n1=5 و n2=0 بفرست، چانک‌ها را فقط برای کانال ۱ بفرست و با CRC درست COMMIT کن.
+گام ۳: پاسخ باید وضعیت 0 باشد؛ برد را ریست کن.
+گام ۴: LUT_READ بگیر: کانال ۱ باید با همان 5 نقطه فعال باشد و کانال ۲ باید فریم صفرنقطه‌ای بدهد (override فلش آن حذف شده باشد).
+گام ۵: در پنل تأیید بگیر که تغییر کانال ۲ «changed-confirmed» است و CRC یا count جای مقادیر واقعی نقاط (counts/BatteryMa) را نگرفته باشد.</t>
         </is>
       </c>
       <c r="F19" s="7" t="inlineStr">
@@ -1989,7 +2035,11 @@
       </c>
       <c r="E20" s="7" t="inlineStr">
         <is>
-          <t>پس از commit reset را درخواست کن؛ یک اجرای flush موفق و یک اجرای flush ناموفق/تزریق‌شده را بررسی کن</t>
+          <t>گام ۱: یک commit موفق (یا commit صفرنقطه‌ای با count=0 معتبر) انجام بده تا grant ریست صادر شود.
+گام ۲: بلافاصله reset را درخواست کن و صبر کن برد بالا بیاید (حداکثر 15 ثانیه).
+گام ۳: از مسیر /t و LUT_READ/LUT_DATA تازه، هر دو کانال و ماندگاری جدول را با مقدار مورد انتظار مقایسه کن؛ هیچ reject یا timeout نباید گزارش شود.
+گام ۴: یک بار هم flush ناموفق را تزریق کن (خطای نوشتن فلش): باید کد CAL_LUT_ST_FLASH برگردد و reset انجام نشود.
+گام ۵: نتیجه بگیر: commit صفرنقطه‌ای بدون جدول فعال پذیرفته می‌شود و reset فقط با grant commit و flush موفق اتفاق می‌افتد.</t>
         </is>
       </c>
       <c r="F20" s="7" t="inlineStr">
@@ -2072,7 +2122,10 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>از پنل LUT را push کن؛ دیالوگ تأیید ریست باید با کادر تیره همرنگ پنل بیاید و Enter تأیید و Esc لغو کند</t>
+          <t>گام ۱: پنل را وصل کن و یک LUT دوکاناله آمادهٔ ارسال داشته باش.
+گام ۲: از پنل LUT را push کن و صبر کن دیالوگ تأیید ریست بیاید.
+گام ۳: دیالوگ باید تیره و هم‌رنگ پنل باشد (#pmod / #121a2c)، نه پنجرهٔ سفید alert ویندوز.
+گام ۴: یک بار کلید Enter را بزن (باید تأیید کند) و یک بار در اجرای بعدی Esc را بزن (باید لغو کند)؛ اگر دو دیالوگ پشت سر هم آمد باید یکی‌یکی در صف PMQ نمایش داده شوند.</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">

</xml_diff>

<commit_message>
docs(validation): split board-performance tests from code/host checks
Per user order each workbook's «برنامه تست» now holds only real board
performance tests. 34 code-level rows (code review, grep checks, host
tools, debugger/stimulus injection, build-flag flips) moved to a new
«تست‌های برنامه‌نویسی» sheet per workbook: Charger 3, Changeover 4,
Diag 2, EspLink 1, Fault 1, Imbalance 1, Jitter 2, Measurement 4,
McuPowerPath 2+2, Protection 3, Rtos 8, Ui 3. CalLut needed none.
Statuses/dates/styles carried over, links rebuilt against the new
sheet/row map (~150 id links), AI_AGENT_RULES records the split.
Documents only; both gates green.

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Firmware/Modules/CalLut/CalLut_Validation.xlsx
+++ b/Firmware/Modules/CalLut/CalLut_Validation.xlsx
@@ -2607,14 +2607,14 @@
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D7" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D14" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D19" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N19" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N20" r:id="rId8"/>
+    <hyperlink ref="D7" location="'برنامه تست'!A6"/>
+    <hyperlink ref="E7" location="'برنامه تست'!A6"/>
+    <hyperlink ref="D14" location="'برنامه تست'!A6"/>
+    <hyperlink ref="E14" location="'برنامه تست'!A6"/>
+    <hyperlink ref="D19" location="'برنامه تست'!A6"/>
+    <hyperlink ref="E19" location="'برنامه تست'!A6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N19" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N20" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>

</xml_diff>